<commit_message>
Updates to incorporate entities of concern requirement from ICCT data
</commit_message>
<xml_diff>
--- a/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
+++ b/InputData/trans/BESP/BAU EV Subsidy Perc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dobrien\Dropbox (Energy Innovation)\Desktop\Models\State Models\eps-newmexico\InputData\trans\BESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3EB6FA-00A5-4BB7-8A3E-0918DC2D352A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9AD7880-2A0F-447F-9863-EA6B33F76573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58740" yWindow="1395" windowWidth="21825" windowHeight="15060" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="61290" yWindow="2610" windowWidth="23100" windowHeight="13305" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId8"/>
+    <pivotCache cacheId="15" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1233,6 +1233,8 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1244,8 +1246,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1294,7 +1294,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44965.855679976848" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Daniel O'Brien" refreshedDate="44993.384917013886" refreshedVersion="8" recordCount="45" xr:uid="{00000000-000A-0000-FFFF-FFFF03000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:P47" sheet="2019 Sales"/>
   </cacheSource>
@@ -2191,7 +2191,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="BAU" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A22:B41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
@@ -2311,7 +2311,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000001000000}" name="BAU 2" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" rowGrandTotals="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G22:J41" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField name="Mfg" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
@@ -3137,7 +3137,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="53">
+      <c r="A46" s="42">
         <v>0.88711067149387013</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -6064,12 +6064,12 @@
     <col min="4" max="34" width="7.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="10">
         <v>2019</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="11">
         <f>BAU!C92</f>
         <v>2745.8606136031603</v>
@@ -6185,72 +6185,95 @@
         <v>1913.0458308533109</v>
       </c>
       <c r="E3" s="11">
-        <v>0</v>
+        <f>BAU!G92</f>
+        <v>1531.9111519939402</v>
       </c>
       <c r="F3" s="11">
-        <v>0</v>
+        <f>BAU!H92</f>
+        <v>1131.4322818029341</v>
       </c>
       <c r="G3" s="11">
-        <v>0</v>
+        <f>BAU!I92</f>
+        <v>933.18813916995919</v>
       </c>
       <c r="H3" s="11">
-        <v>0</v>
+        <f>BAU!J92</f>
+        <v>933.18813916995953</v>
       </c>
       <c r="I3" s="11">
-        <v>0</v>
+        <f>BAU!K92</f>
+        <v>744.00735890914916</v>
       </c>
       <c r="J3" s="11">
-        <v>0</v>
+        <f>BAU!L92</f>
+        <v>744.00735890914984</v>
       </c>
       <c r="K3" s="11">
-        <v>0</v>
+        <f>BAU!M92</f>
+        <v>621.92251501542137</v>
       </c>
       <c r="L3" s="11">
-        <v>0</v>
+        <f>BAU!N92</f>
+        <v>240.24673989502756</v>
       </c>
       <c r="M3" s="11">
-        <v>0</v>
+        <f>BAU!O92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="N3" s="11">
-        <v>0</v>
+        <f>BAU!P92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="O3" s="11">
-        <v>0</v>
+        <f>BAU!Q92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="P3" s="11">
-        <v>0</v>
+        <f>BAU!R92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q3" s="11">
-        <v>0</v>
+        <f>BAU!S92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="R3" s="11">
-        <v>0</v>
+        <f>BAU!T92</f>
+        <v>18.397272874844433</v>
       </c>
       <c r="S3" s="11">
-        <v>0</v>
+        <f>BAU!U92</f>
+        <v>18.397272874844436</v>
       </c>
       <c r="T3" s="11">
+        <f>BAU!V92</f>
         <v>0</v>
       </c>
       <c r="U3" s="11">
+        <f>BAU!W92</f>
         <v>0</v>
       </c>
       <c r="V3" s="11">
+        <f>BAU!X92</f>
         <v>0</v>
       </c>
       <c r="W3" s="11">
+        <f>BAU!Y92</f>
         <v>0</v>
       </c>
       <c r="X3" s="11">
+        <f>BAU!Z92</f>
         <v>0</v>
       </c>
       <c r="Y3" s="11">
+        <f>BAU!AA92</f>
         <v>0</v>
       </c>
       <c r="Z3" s="11">
+        <f>BAU!AB92</f>
         <v>0</v>
       </c>
       <c r="AA3" s="11">
+        <f>BAU!AC92</f>
         <v>0</v>
       </c>
       <c r="AB3" s="11">
@@ -6273,29 +6296,30 @@
         <f>BAU!AH92</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="AG3" s="11"/>
+    </row>
+    <row r="4" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="31"/>
       <c r="E4" s="40" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="32" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="31" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" s="31" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="32" t="s">
         <v>132</v>
       </c>
@@ -6306,7 +6330,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A9" s="31">
         <v>2500</v>
       </c>
@@ -6317,7 +6341,7 @@
         <v>39250017</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="31">
         <v>5000</v>
       </c>
@@ -6328,7 +6352,7 @@
         <v>5540545</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="31">
         <v>3500</v>
       </c>
@@ -6339,7 +6363,7 @@
         <v>952065</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" s="33">
         <v>1500</v>
       </c>
@@ -6350,7 +6374,7 @@
         <v>4681666</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="31">
         <v>2500</v>
       </c>
@@ -6361,7 +6385,7 @@
         <v>6811779</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="31">
         <v>1500</v>
       </c>
@@ -6372,7 +6396,7 @@
         <v>3923561</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="31">
         <v>2500</v>
       </c>
@@ -6383,7 +6407,7 @@
         <v>1056426</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:33" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" s="34" t="s">
         <v>134</v>
       </c>
@@ -6993,63 +7017,63 @@
       </c>
       <c r="E33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1531.9111519939402</v>
       </c>
       <c r="F33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1131.4322818029341</v>
       </c>
       <c r="G33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>933.18813916995919</v>
       </c>
       <c r="H33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>933.18813916995953</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>744.00735890914916</v>
       </c>
       <c r="J33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>744.00735890914984</v>
       </c>
       <c r="K33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>621.92251501542137</v>
       </c>
       <c r="L33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>240.24673989502756</v>
       </c>
       <c r="M33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="N33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="O33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="P33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="Q33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="R33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844433</v>
       </c>
       <c r="S33" s="12">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>18.397272874844436</v>
       </c>
       <c r="T33" s="12">
         <f t="shared" si="2"/>
@@ -11263,13 +11287,13 @@
       <c r="G24" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="H24" s="44">
+      <c r="H24" s="46">
         <v>175</v>
       </c>
-      <c r="I24" s="45">
+      <c r="I24" s="47">
         <v>210</v>
       </c>
-      <c r="J24" s="46">
+      <c r="J24" s="48">
         <v>45</v>
       </c>
       <c r="K24" s="8">
@@ -11287,13 +11311,13 @@
       <c r="G25" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="47">
+      <c r="H25" s="49">
         <v>997</v>
       </c>
-      <c r="I25" s="48">
+      <c r="I25" s="50">
         <v>1111</v>
       </c>
-      <c r="J25" s="49">
+      <c r="J25" s="51">
         <v>1147</v>
       </c>
       <c r="K25" s="8">
@@ -11311,13 +11335,13 @@
       <c r="G26" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="H26" s="47">
+      <c r="H26" s="49">
         <v>72</v>
       </c>
-      <c r="I26" s="48">
+      <c r="I26" s="50">
         <v>87</v>
       </c>
-      <c r="J26" s="49">
+      <c r="J26" s="51">
         <v>33</v>
       </c>
       <c r="K26" s="8">
@@ -11335,13 +11359,13 @@
       <c r="G27" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="H27" s="47">
+      <c r="H27" s="49">
         <v>557</v>
       </c>
-      <c r="I27" s="48">
+      <c r="I27" s="50">
         <v>573</v>
       </c>
-      <c r="J27" s="49">
+      <c r="J27" s="51">
         <v>611</v>
       </c>
       <c r="K27" s="8">
@@ -11359,13 +11383,13 @@
       <c r="G28" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H28" s="47">
+      <c r="H28" s="49">
         <v>2044</v>
       </c>
-      <c r="I28" s="48">
+      <c r="I28" s="50">
         <v>2430</v>
       </c>
-      <c r="J28" s="49">
+      <c r="J28" s="51">
         <v>3782</v>
       </c>
       <c r="K28" s="8">
@@ -11383,13 +11407,13 @@
       <c r="G29" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="H29" s="47">
+      <c r="H29" s="49">
         <v>1270</v>
       </c>
-      <c r="I29" s="48">
+      <c r="I29" s="50">
         <v>1281</v>
       </c>
-      <c r="J29" s="49">
+      <c r="J29" s="51">
         <v>1403</v>
       </c>
       <c r="K29" s="8">
@@ -11407,13 +11431,13 @@
       <c r="G30" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="H30" s="47">
+      <c r="H30" s="49">
         <v>111</v>
       </c>
-      <c r="I30" s="48">
+      <c r="I30" s="50">
         <v>173</v>
       </c>
-      <c r="J30" s="49">
+      <c r="J30" s="51">
         <v>256</v>
       </c>
       <c r="K30" s="8">
@@ -11431,13 +11455,13 @@
       <c r="G31" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="H31" s="47">
+      <c r="H31" s="49">
         <v>210</v>
       </c>
-      <c r="I31" s="48">
+      <c r="I31" s="50">
         <v>186</v>
       </c>
-      <c r="J31" s="49">
+      <c r="J31" s="51">
         <v>212</v>
       </c>
       <c r="K31" s="8">
@@ -11455,13 +11479,13 @@
       <c r="G32" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="H32" s="47">
+      <c r="H32" s="49">
         <v>309</v>
       </c>
-      <c r="I32" s="48">
+      <c r="I32" s="50">
         <v>517</v>
       </c>
-      <c r="J32" s="49">
+      <c r="J32" s="51">
         <v>240</v>
       </c>
       <c r="K32" s="8">
@@ -11479,13 +11503,13 @@
       <c r="G33" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="H33" s="47">
+      <c r="H33" s="49">
         <v>398</v>
       </c>
-      <c r="I33" s="48">
+      <c r="I33" s="50">
         <v>382</v>
       </c>
-      <c r="J33" s="49">
+      <c r="J33" s="51">
         <v>532</v>
       </c>
       <c r="K33" s="8">
@@ -11503,13 +11527,13 @@
       <c r="G34" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H34" s="47">
+      <c r="H34" s="49">
         <v>133</v>
       </c>
-      <c r="I34" s="48">
+      <c r="I34" s="50">
         <v>157</v>
       </c>
-      <c r="J34" s="49">
+      <c r="J34" s="51">
         <v>341</v>
       </c>
       <c r="K34" s="8">
@@ -11527,13 +11551,13 @@
       <c r="G35" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="H35" s="47">
+      <c r="H35" s="49">
         <v>717</v>
       </c>
-      <c r="I35" s="48">
+      <c r="I35" s="50">
         <v>654</v>
       </c>
-      <c r="J35" s="49">
+      <c r="J35" s="51">
         <v>1314</v>
       </c>
       <c r="K35" s="8">
@@ -11551,13 +11575,13 @@
       <c r="G36" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="H36" s="47">
+      <c r="H36" s="49">
         <v>215</v>
       </c>
-      <c r="I36" s="48">
+      <c r="I36" s="50">
         <v>255</v>
       </c>
-      <c r="J36" s="49">
+      <c r="J36" s="51">
         <v>310</v>
       </c>
       <c r="K36" s="8">
@@ -11575,11 +11599,11 @@
       <c r="G37" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="H37" s="47"/>
-      <c r="I37" s="48">
+      <c r="H37" s="49"/>
+      <c r="I37" s="50">
         <v>27</v>
       </c>
-      <c r="J37" s="49">
+      <c r="J37" s="51">
         <v>52</v>
       </c>
       <c r="K37" s="8">
@@ -11597,13 +11621,13 @@
       <c r="G38" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="H38" s="47">
+      <c r="H38" s="49">
         <v>8000</v>
       </c>
-      <c r="I38" s="48">
+      <c r="I38" s="50">
         <v>7275</v>
       </c>
-      <c r="J38" s="49">
+      <c r="J38" s="51">
         <v>14625</v>
       </c>
       <c r="K38" s="8">
@@ -11621,13 +11645,13 @@
       <c r="G39" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="H39" s="47">
+      <c r="H39" s="49">
         <v>1123</v>
       </c>
-      <c r="I39" s="48">
+      <c r="I39" s="50">
         <v>1205</v>
       </c>
-      <c r="J39" s="49">
+      <c r="J39" s="51">
         <v>1820</v>
       </c>
       <c r="K39" s="8">
@@ -11645,13 +11669,13 @@
       <c r="G40" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="H40" s="47">
+      <c r="H40" s="49">
         <v>220</v>
       </c>
-      <c r="I40" s="48">
+      <c r="I40" s="50">
         <v>250</v>
       </c>
-      <c r="J40" s="49">
+      <c r="J40" s="51">
         <v>335</v>
       </c>
       <c r="K40" s="8">
@@ -11669,13 +11693,13 @@
       <c r="G41" s="25" t="s">
         <v>175</v>
       </c>
-      <c r="H41" s="50">
+      <c r="H41" s="52">
         <v>164</v>
       </c>
-      <c r="I41" s="51">
+      <c r="I41" s="53">
         <v>118</v>
       </c>
-      <c r="J41" s="52">
+      <c r="J41" s="54">
         <v>581</v>
       </c>
       <c r="K41" s="8">
@@ -20399,7 +20423,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="44" t="s">
         <v>262</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -20413,7 +20437,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="43"/>
+      <c r="A2" s="45"/>
       <c r="B2" s="8" t="s">
         <v>266</v>
       </c>
@@ -20425,7 +20449,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="43"/>
+      <c r="A3" s="45"/>
       <c r="C3" s="8">
         <v>200000</v>
       </c>
@@ -20434,7 +20458,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="43"/>
+      <c r="A4" s="45"/>
       <c r="D4" s="8">
         <v>200000</v>
       </c>
@@ -21791,15 +21815,15 @@
       <c r="A2" s="8" t="s">
         <v>273</v>
       </c>
-      <c r="B2" s="54">
+      <c r="B2" s="43">
         <f>C2</f>
         <v>2435.88225276207</v>
       </c>
-      <c r="C2" s="54">
+      <c r="C2" s="43">
         <f>D2</f>
         <v>2435.88225276207</v>
       </c>
-      <c r="D2" s="54">
+      <c r="D2" s="43">
         <f>E2</f>
         <v>2435.88225276207</v>
       </c>
@@ -21821,63 +21845,63 @@
       </c>
       <c r="I2" s="12">
         <f>Data!E33*About!$A46</f>
-        <v>0</v>
+        <v>1358.9747307142925</v>
       </c>
       <c r="J2" s="12">
         <f>Data!F33*About!$A46</f>
-        <v>0</v>
+        <v>1003.7056512600426</v>
       </c>
       <c r="K2" s="12">
         <f>Data!G33*About!$A46</f>
-        <v>0</v>
+        <v>827.84115676917759</v>
       </c>
       <c r="L2" s="12">
         <f>Data!H33*About!$A46</f>
-        <v>0</v>
+        <v>827.84115676917793</v>
       </c>
       <c r="M2" s="12">
         <f>Data!I33*About!$A46</f>
-        <v>0</v>
+        <v>660.01686775827613</v>
       </c>
       <c r="N2" s="12">
         <f>Data!J33*About!$A46</f>
-        <v>0</v>
+        <v>660.0168677582767</v>
       </c>
       <c r="O2" s="12">
         <f>Data!K33*About!$A46</f>
-        <v>0</v>
+        <v>551.71409991248697</v>
       </c>
       <c r="P2" s="12">
         <f>Data!L33*About!$A46</f>
-        <v>0</v>
+        <v>213.12544675249106</v>
       </c>
       <c r="Q2" s="12">
         <f>Data!M33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="R2" s="12">
         <f>Data!N33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="S2" s="12">
         <f>Data!O33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="T2" s="12">
         <f>Data!P33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="U2" s="12">
         <f>Data!Q33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="V2" s="12">
         <f>Data!R33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659206</v>
       </c>
       <c r="W2" s="12">
         <f>Data!S33*About!$A46</f>
-        <v>0</v>
+        <v>16.320417093659209</v>
       </c>
       <c r="X2" s="12">
         <f>Data!T33*About!$A46</f>

</xml_diff>